<commit_message>
Adding the boat launches to the map
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/survey_dates.xlsx
+++ b/Jones_honours/01_raw_data/survey_dates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D88A572-A415-3841-989E-4ADE40FBFF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29BDBA22-9223-2847-8BA6-1B9B9F47F95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27640" yWindow="4100" windowWidth="27240" windowHeight="16440" xr2:uid="{1E870310-51C7-2A49-81D3-0EC67314724B}"/>
+    <workbookView xWindow="-27640" yWindow="4100" windowWidth="27240" windowHeight="16140" xr2:uid="{1E870310-51C7-2A49-81D3-0EC67314724B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>